<commit_message>
core: 左右链支持按炮区人工指定 + tune_chains 贪心标定（1003 0.883→0.913/+6.6%→+0.2%、0915→0.922、1004→0.805）
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/_批量汇总/批量汇总.xlsx
+++ b/北部山头3940平台2026/7、单日数据/_批量汇总/批量汇总.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,19 +480,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>282.905</v>
+        <v>290.37</v>
       </c>
       <c r="E2" t="n">
-        <v>3111.952</v>
+        <v>3194.073</v>
       </c>
       <c r="F2" t="n">
-        <v>8402.27</v>
+        <v>8623.998</v>
       </c>
       <c r="G2" t="n">
         <v>1.76</v>
       </c>
       <c r="H2" t="n">
-        <v>147.88</v>
+        <v>151.782</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>76.89700000000001</v>
+        <v>73.786</v>
       </c>
       <c r="E4" t="n">
-        <v>768.967</v>
+        <v>737.86</v>
       </c>
       <c r="F4" t="n">
-        <v>2076.212</v>
+        <v>1992.223</v>
       </c>
       <c r="G4" t="n">
         <v>1.825</v>
       </c>
       <c r="H4" t="n">
-        <v>37.891</v>
+        <v>36.358</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -620,19 +620,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>662.068</v>
+        <v>664.117</v>
       </c>
       <c r="E6" t="n">
-        <v>6492.225</v>
+        <v>6513.236</v>
       </c>
       <c r="F6" t="n">
-        <v>17529.007</v>
+        <v>17585.738</v>
       </c>
       <c r="G6" t="n">
         <v>1.263</v>
       </c>
       <c r="H6" t="n">
-        <v>221.351</v>
+        <v>222.067</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -830,23 +830,23 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>614.933</v>
+        <v>638.4880000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>6861.985</v>
+        <v>7121.053</v>
       </c>
       <c r="F12" t="n">
-        <v>18527.359</v>
+        <v>19226.842</v>
       </c>
       <c r="G12" t="n">
-        <v>2.101</v>
+        <v>2.004</v>
       </c>
       <c r="H12" t="n">
-        <v>389.336</v>
+        <v>385.273</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>P38、P36、P33、P12、P30、P34、P29、P19、P18、P31、P23、P14、P1、P32、P16、P9、P26、P11、P21、P28、P27、P15、P8、P35、P37、P22</t>
+          <t>P38、P36、P33、P12、P30、P34、P29、P19、P18、P31、P23、P14、P1、P32、P16、P9、P26、P11、P21、P28、P27、P15、P8、P35、P25、P37、P24、P22、P20</t>
         </is>
       </c>
     </row>
@@ -865,19 +865,19 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>212.457</v>
+        <v>212.304</v>
       </c>
       <c r="E13" t="n">
-        <v>2337.028</v>
+        <v>2335.348</v>
       </c>
       <c r="F13" t="n">
-        <v>6309.976</v>
+        <v>6305.438</v>
       </c>
       <c r="G13" t="n">
         <v>1.099</v>
       </c>
       <c r="H13" t="n">
-        <v>69.34</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -888,35 +888,35 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.000-1.500</t>
+          <t>1.500-3.000</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>78.309</v>
+        <v>83.342</v>
       </c>
       <c r="E14" t="n">
-        <v>861.396</v>
+        <v>916.763</v>
       </c>
       <c r="F14" t="n">
-        <v>2325.768</v>
+        <v>2475.259</v>
       </c>
       <c r="G14" t="n">
-        <v>1.143</v>
+        <v>1.545</v>
       </c>
       <c r="H14" t="n">
-        <v>26.591</v>
+        <v>38.243</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>P25、P24、P20</t>
+          <t>P30、P28</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -935,23 +935,23 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>83.342</v>
+        <v>89.502</v>
       </c>
       <c r="E15" t="n">
-        <v>916.763</v>
+        <v>895.016</v>
       </c>
       <c r="F15" t="n">
-        <v>2475.259</v>
+        <v>2416.545</v>
       </c>
       <c r="G15" t="n">
-        <v>1.545</v>
+        <v>2.18</v>
       </c>
       <c r="H15" t="n">
-        <v>38.243</v>
+        <v>52.681</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>P30、P28</t>
+          <t>P3、P2、P1</t>
         </is>
       </c>
     </row>
@@ -962,31 +962,31 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.500-3.000</t>
+          <t>1.000-1.500</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>89.502</v>
+        <v>78.16800000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>895.016</v>
+        <v>781.682</v>
       </c>
       <c r="F16" t="n">
-        <v>2416.545</v>
+        <v>2110.541</v>
       </c>
       <c r="G16" t="n">
-        <v>2.18</v>
+        <v>1.375</v>
       </c>
       <c r="H16" t="n">
-        <v>52.681</v>
+        <v>29.02</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>P3、P2、P1</t>
+          <t>P6、P4</t>
         </is>
       </c>
     </row>
@@ -997,66 +997,66 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.000-1.500</t>
+          <t>0.500-1.000</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>78.67100000000001</v>
+        <v>672.726</v>
       </c>
       <c r="E17" t="n">
-        <v>786.705</v>
+        <v>7325.304</v>
       </c>
       <c r="F17" t="n">
-        <v>2124.105</v>
+        <v>19778.32</v>
       </c>
       <c r="G17" t="n">
-        <v>1.375</v>
+        <v>0.82</v>
       </c>
       <c r="H17" t="n">
-        <v>29.206</v>
+        <v>162.25</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>P6、P4</t>
+          <t>P8、P11、P5、P7、P20、P23、P26、P14、P12、P10、P29、P27、P9、P31、P21、P13</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.500-1.000</t>
+          <t>1.000-1.500</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>685.884</v>
+        <v>163.263</v>
       </c>
       <c r="E18" t="n">
-        <v>7469.899</v>
+        <v>1897.084</v>
       </c>
       <c r="F18" t="n">
-        <v>20168.728</v>
+        <v>5122.126</v>
       </c>
       <c r="G18" t="n">
-        <v>0.82</v>
+        <v>1.204</v>
       </c>
       <c r="H18" t="n">
-        <v>165.453</v>
+        <v>61.688</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>P8、P11、P5、P7、P20、P23、P26、P14、P12、P10、P29、P27、P9、P31、P21、P13</t>
+          <t>P2、P3、P5、P12、P1、P7</t>
         </is>
       </c>
     </row>
@@ -1067,31 +1067,31 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.000-1.500</t>
+          <t>0.500-1.000</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>163.263</v>
+        <v>114.812</v>
       </c>
       <c r="E19" t="n">
-        <v>1897.084</v>
+        <v>1322.7</v>
       </c>
       <c r="F19" t="n">
-        <v>5122.126</v>
+        <v>3571.291</v>
       </c>
       <c r="G19" t="n">
-        <v>1.204</v>
+        <v>0.729</v>
       </c>
       <c r="H19" t="n">
-        <v>61.688</v>
+        <v>26.039</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>P2、P3、P5、P12、P1、P7</t>
+          <t>P4、P9、P6、P8</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1110,56 +1110,21 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>114.812</v>
+        <v>59.367</v>
       </c>
       <c r="E20" t="n">
-        <v>1322.7</v>
+        <v>653.039</v>
       </c>
       <c r="F20" t="n">
-        <v>3571.291</v>
+        <v>1763.206</v>
       </c>
       <c r="G20" t="n">
-        <v>0.729</v>
+        <v>0.68</v>
       </c>
       <c r="H20" t="n">
-        <v>26.039</v>
+        <v>11.99</v>
       </c>
       <c r="I20" t="inlineStr">
-        <is>
-          <t>P4、P9、P6、P8</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1008</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>3</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>0.500-1.000</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>59.367</v>
-      </c>
-      <c r="E21" t="n">
-        <v>653.039</v>
-      </c>
-      <c r="F21" t="n">
-        <v>1763.206</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H21" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="I21" t="inlineStr">
         <is>
           <t>P23、P14</t>
         </is>
@@ -1224,13 +1189,13 @@
         <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>12995.756</v>
+        <v>13067.782</v>
       </c>
       <c r="E2" t="n">
-        <v>35088.54</v>
+        <v>35283.01</v>
       </c>
       <c r="F2" t="n">
-        <v>531.426</v>
+        <v>534.5119999999999</v>
       </c>
     </row>
     <row r="3">
@@ -1265,16 +1230,16 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>10060.408</v>
+        <v>9456.4</v>
       </c>
       <c r="E4" t="n">
-        <v>27163.103</v>
+        <v>25532.28</v>
       </c>
       <c r="F4" t="n">
-        <v>485.266</v>
+        <v>454.562</v>
       </c>
     </row>
     <row r="5">
@@ -1290,13 +1255,13 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>10068.384</v>
+        <v>9918.764999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>27184.637</v>
+        <v>26780.665</v>
       </c>
       <c r="F5" t="n">
-        <v>285.583</v>
+        <v>282.194</v>
       </c>
     </row>
     <row r="6">
@@ -1435,7 +1400,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>1 个矿孔原本落在矿界外（P19）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: 0922 标定后数值更新（-13.1%）+ --by-volume 用法
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/_批量汇总/批量汇总.xlsx
+++ b/北部山头3940平台2026/7、单日数据/_批量汇总/批量汇总.xlsx
@@ -690,19 +690,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>214.958</v>
+        <v>219.368</v>
       </c>
       <c r="E8" t="n">
-        <v>891.783</v>
+        <v>897.282</v>
       </c>
       <c r="F8" t="n">
-        <v>2407.815</v>
+        <v>2422.661</v>
       </c>
       <c r="G8" t="n">
         <v>1.727</v>
       </c>
       <c r="H8" t="n">
-        <v>41.575</v>
+        <v>41.831</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>338.579</v>
+        <v>365.364</v>
       </c>
       <c r="E9" t="n">
-        <v>1196.277</v>
+        <v>1292.135</v>
       </c>
       <c r="F9" t="n">
-        <v>3229.947</v>
+        <v>3488.765</v>
       </c>
       <c r="G9" t="n">
         <v>1.333</v>
       </c>
       <c r="H9" t="n">
-        <v>43.051</v>
+        <v>46.5</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -760,19 +760,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>283.012</v>
+        <v>297.081</v>
       </c>
       <c r="E10" t="n">
-        <v>3047.971</v>
+        <v>3199.778</v>
       </c>
       <c r="F10" t="n">
-        <v>8229.522999999999</v>
+        <v>8639.401</v>
       </c>
       <c r="G10" t="n">
         <v>0.824</v>
       </c>
       <c r="H10" t="n">
-        <v>67.788</v>
+        <v>71.16500000000001</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -795,19 +795,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>339.922</v>
+        <v>395.866</v>
       </c>
       <c r="E11" t="n">
-        <v>661.559</v>
+        <v>759.133</v>
       </c>
       <c r="F11" t="n">
-        <v>1786.21</v>
+        <v>2049.658</v>
       </c>
       <c r="G11" t="n">
         <v>0.695</v>
       </c>
       <c r="H11" t="n">
-        <v>12.414</v>
+        <v>14.245</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1176,13 +1176,13 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>5797.591</v>
+        <v>6148.327</v>
       </c>
       <c r="E3" t="n">
-        <v>15653.494</v>
+        <v>16600.484</v>
       </c>
       <c r="F3" t="n">
-        <v>164.828</v>
+        <v>173.741</v>
       </c>
     </row>
     <row r="4">
@@ -1328,7 +1328,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
         <v>15</v>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2 个矿孔原本落在矿界外（BL1、BL6）；3 个矿孔原本落在矿界外（P9、P15、P17）</t>
+          <t>矿界原本碎成 2 片；2 个矿孔原本落在矿界外（BL1、BL6）；3 个矿孔原本落在矿界外（P9、P15、P17）</t>
         </is>
       </c>
     </row>

</xml_diff>